<commit_message>
TallyOne 1.9 - purge previous-voyage leftovers baked into tally templates, merge seal-list container cell, tidy header alignment and row heights
</commit_message>
<xml_diff>
--- a/dist/tally_templates/ATPR.xlsx
+++ b/dist/tally_templates/ATPR.xlsx
@@ -1150,7 +1150,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac x16r2">
   <numFmts count="9">
     <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * -#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* (#,##0);_(* &quot;-&quot;_);_(@_)"/>
@@ -3167,7 +3167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="544">
+  <cellXfs count="573">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -4779,6 +4779,93 @@
     </xf>
     <xf numFmtId="172" fontId="10" fillId="0" borderId="129" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="109" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="110" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="109" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="109" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="120" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="91" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="122" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4787,11 +4874,11 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <ns3:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <ns4:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -5059,7 +5146,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Y145"/>
   <sheetFormatPr defaultRowHeight="17.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
@@ -5821,14 +5908,14 @@
       <c r="D7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="206" t="s">
+      <c r="E7" s="208" t="s">
         <v>61</v>
       </c>
       <c r="F7" s="206"/>
       <c r="G7" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="207">
+      <c r="H7" s="560">
         <v>46229</v>
       </c>
       <c r="I7" s="8"/>
@@ -5858,14 +5945,14 @@
       <c r="D8" s="334" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="208">
         <v>16</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" s="208" t="s">
         <v>95</v>
       </c>
       <c r="I8" s="8"/>
@@ -7175,14 +7262,14 @@
       <c r="D55" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E55" s="206" t="s">
+      <c r="E55" s="208" t="s">
         <v>61</v>
       </c>
       <c r="F55" s="206"/>
       <c r="G55" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="H55" s="207">
+      <c r="H55" s="560">
         <v>46229</v>
       </c>
       <c r="I55" s="8"/>
@@ -7212,14 +7299,14 @@
       <c r="D56" s="334" t="s">
         <v>7</v>
       </c>
-      <c r="E56" s="8">
+      <c r="E56" s="208">
         <v>16</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="H56" s="8" t="s">
+      <c r="H56" s="208" t="s">
         <v>95</v>
       </c>
       <c r="I56" s="8"/>
@@ -7344,27 +7431,17 @@
       <c r="Y59" s="105"/>
     </row>
     <row r="60" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="54" t="s">
-        <v>108</v>
-      </c>
+      <c r="A60" s="54"/>
       <c r="B60" s="342"/>
-      <c r="C60" s="342" t="s">
-        <v>109</v>
-      </c>
+      <c r="C60" s="342"/>
       <c r="D60" s="185"/>
       <c r="E60" s="57"/>
-      <c r="F60" s="343">
-        <v>-18</v>
-      </c>
-      <c r="G60" s="343">
-        <v>-17.3</v>
-      </c>
+      <c r="F60" s="343"/>
+      <c r="G60" s="343"/>
       <c r="H60" s="344" t="s">
         <v>110</v>
       </c>
-      <c r="I60" s="54" t="s">
-        <v>111</v>
-      </c>
+      <c r="I60" s="54"/>
       <c r="J60" s="41"/>
       <c r="K60" s="41"/>
       <c r="L60" s="41"/>
@@ -7383,27 +7460,15 @@
       <c r="Y60" s="41"/>
     </row>
     <row r="61" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="233" t="s">
-        <v>112</v>
-      </c>
+      <c r="A61" s="233"/>
       <c r="B61" s="346"/>
-      <c r="C61" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C61" s="346"/>
       <c r="D61" s="226"/>
       <c r="E61" s="177"/>
-      <c r="F61" s="347">
-        <v>-2.5</v>
-      </c>
-      <c r="G61" s="347">
-        <v>-2.5</v>
-      </c>
-      <c r="H61" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I61" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F61" s="347"/>
+      <c r="G61" s="347"/>
+      <c r="H61" s="348"/>
+      <c r="I61" s="233"/>
       <c r="J61" s="41"/>
       <c r="K61" s="41"/>
       <c r="L61" s="41"/>
@@ -7422,27 +7487,15 @@
       <c r="Y61" s="41"/>
     </row>
     <row r="62" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="233" t="s">
-        <v>114</v>
-      </c>
+      <c r="A62" s="233"/>
       <c r="B62" s="346"/>
-      <c r="C62" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C62" s="346"/>
       <c r="D62" s="226"/>
       <c r="E62" s="177"/>
-      <c r="F62" s="347">
-        <v>-18</v>
-      </c>
-      <c r="G62" s="347">
-        <v>-23.3</v>
-      </c>
-      <c r="H62" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I62" s="233" t="s">
-        <v>115</v>
-      </c>
+      <c r="F62" s="347"/>
+      <c r="G62" s="347"/>
+      <c r="H62" s="348"/>
+      <c r="I62" s="233"/>
       <c r="J62" s="41"/>
       <c r="K62" s="41"/>
       <c r="L62" s="41"/>
@@ -7461,27 +7514,15 @@
       <c r="Y62" s="41"/>
     </row>
     <row r="63" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="233" t="s">
-        <v>116</v>
-      </c>
+      <c r="A63" s="233"/>
       <c r="B63" s="346"/>
-      <c r="C63" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C63" s="346"/>
       <c r="D63" s="226"/>
       <c r="E63" s="177"/>
-      <c r="F63" s="347">
-        <v>-2.5</v>
-      </c>
-      <c r="G63" s="347">
-        <v>-2.5</v>
-      </c>
-      <c r="H63" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I63" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F63" s="347"/>
+      <c r="G63" s="347"/>
+      <c r="H63" s="348"/>
+      <c r="I63" s="233"/>
       <c r="J63" s="41"/>
       <c r="K63" s="41"/>
       <c r="L63" s="41"/>
@@ -7500,27 +7541,15 @@
       <c r="Y63" s="41"/>
     </row>
     <row r="64" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="299" t="s">
-        <v>117</v>
-      </c>
+      <c r="A64" s="299"/>
       <c r="B64" s="350"/>
-      <c r="C64" s="350" t="s">
-        <v>109</v>
-      </c>
+      <c r="C64" s="350"/>
       <c r="D64" s="172"/>
       <c r="E64" s="173"/>
-      <c r="F64" s="351">
-        <v>-18</v>
-      </c>
-      <c r="G64" s="351">
-        <v>-22.3</v>
-      </c>
-      <c r="H64" s="352" t="s">
-        <v>113</v>
-      </c>
-      <c r="I64" s="299" t="s">
-        <v>111</v>
-      </c>
+      <c r="F64" s="351"/>
+      <c r="G64" s="351"/>
+      <c r="H64" s="352"/>
+      <c r="I64" s="299"/>
       <c r="J64" s="41"/>
       <c r="K64" s="41"/>
       <c r="L64" s="41"/>
@@ -7539,27 +7568,15 @@
       <c r="Y64" s="41"/>
     </row>
     <row r="65" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="54" t="s">
-        <v>118</v>
-      </c>
+      <c r="A65" s="54"/>
       <c r="B65" s="342"/>
-      <c r="C65" s="342" t="s">
-        <v>109</v>
-      </c>
+      <c r="C65" s="342"/>
       <c r="D65" s="185"/>
       <c r="E65" s="57"/>
-      <c r="F65" s="353">
-        <v>-25</v>
-      </c>
-      <c r="G65" s="353">
-        <v>-28</v>
-      </c>
-      <c r="H65" s="344" t="s">
-        <v>113</v>
-      </c>
-      <c r="I65" s="54" t="s">
-        <v>111</v>
-      </c>
+      <c r="F65" s="353"/>
+      <c r="G65" s="353"/>
+      <c r="H65" s="344"/>
+      <c r="I65" s="54"/>
       <c r="J65" s="41"/>
       <c r="K65" s="41"/>
       <c r="L65" s="41"/>
@@ -7578,27 +7595,15 @@
       <c r="Y65" s="41"/>
     </row>
     <row r="66" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="233" t="s">
-        <v>119</v>
-      </c>
+      <c r="A66" s="233"/>
       <c r="B66" s="346"/>
-      <c r="C66" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C66" s="346"/>
       <c r="D66" s="226"/>
       <c r="E66" s="177"/>
-      <c r="F66" s="354">
-        <v>-25</v>
-      </c>
-      <c r="G66" s="354">
-        <v>-25.5</v>
-      </c>
-      <c r="H66" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I66" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F66" s="354"/>
+      <c r="G66" s="354"/>
+      <c r="H66" s="348"/>
+      <c r="I66" s="233"/>
       <c r="J66" s="41"/>
       <c r="K66" s="41"/>
       <c r="L66" s="41"/>
@@ -7617,27 +7622,15 @@
       <c r="Y66" s="41"/>
     </row>
     <row r="67" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="233" t="s">
-        <v>120</v>
-      </c>
+      <c r="A67" s="233"/>
       <c r="B67" s="346"/>
-      <c r="C67" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C67" s="346"/>
       <c r="D67" s="226"/>
       <c r="E67" s="177"/>
-      <c r="F67" s="347">
-        <v>-2.5</v>
-      </c>
-      <c r="G67" s="347">
-        <v>-2.5</v>
-      </c>
-      <c r="H67" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I67" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F67" s="347"/>
+      <c r="G67" s="347"/>
+      <c r="H67" s="348"/>
+      <c r="I67" s="233"/>
       <c r="J67" s="41"/>
       <c r="K67" s="41"/>
       <c r="L67" s="41"/>
@@ -7656,27 +7649,15 @@
       <c r="Y67" s="41"/>
     </row>
     <row r="68" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="233" t="s">
-        <v>121</v>
-      </c>
+      <c r="A68" s="233"/>
       <c r="B68" s="346"/>
-      <c r="C68" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C68" s="346"/>
       <c r="D68" s="226"/>
       <c r="E68" s="177"/>
-      <c r="F68" s="354">
-        <v>-18</v>
-      </c>
-      <c r="G68" s="347">
-        <v>-21.9</v>
-      </c>
-      <c r="H68" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I68" s="233" t="s">
-        <v>115</v>
-      </c>
+      <c r="F68" s="354"/>
+      <c r="G68" s="347"/>
+      <c r="H68" s="348"/>
+      <c r="I68" s="233"/>
       <c r="J68" s="41"/>
       <c r="K68" s="41"/>
       <c r="L68" s="41"/>
@@ -7695,27 +7676,15 @@
       <c r="Y68" s="41"/>
     </row>
     <row r="69" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="299" t="s">
-        <v>122</v>
-      </c>
+      <c r="A69" s="299"/>
       <c r="B69" s="350"/>
-      <c r="C69" s="350" t="s">
-        <v>109</v>
-      </c>
+      <c r="C69" s="350"/>
       <c r="D69" s="172"/>
       <c r="E69" s="173"/>
-      <c r="F69" s="351">
-        <v>-18</v>
-      </c>
-      <c r="G69" s="351">
-        <v>-24</v>
-      </c>
-      <c r="H69" s="352" t="s">
-        <v>113</v>
-      </c>
-      <c r="I69" s="299" t="s">
-        <v>115</v>
-      </c>
+      <c r="F69" s="351"/>
+      <c r="G69" s="351"/>
+      <c r="H69" s="352"/>
+      <c r="I69" s="299"/>
       <c r="J69" s="41"/>
       <c r="K69" s="41"/>
       <c r="L69" s="41"/>
@@ -7734,27 +7703,15 @@
       <c r="Y69" s="41"/>
     </row>
     <row r="70" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="54" t="s">
-        <v>123</v>
-      </c>
+      <c r="A70" s="54"/>
       <c r="B70" s="342"/>
-      <c r="C70" s="342" t="s">
-        <v>109</v>
-      </c>
+      <c r="C70" s="342"/>
       <c r="D70" s="252"/>
       <c r="E70" s="253"/>
-      <c r="F70" s="355">
-        <v>0</v>
-      </c>
-      <c r="G70" s="355">
-        <v>0</v>
-      </c>
-      <c r="H70" s="344" t="s">
-        <v>113</v>
-      </c>
-      <c r="I70" s="54" t="s">
-        <v>115</v>
-      </c>
+      <c r="F70" s="355"/>
+      <c r="G70" s="355"/>
+      <c r="H70" s="344"/>
+      <c r="I70" s="54"/>
       <c r="J70" s="41"/>
       <c r="K70" s="41"/>
       <c r="L70" s="41"/>
@@ -7773,27 +7730,15 @@
       <c r="Y70" s="41"/>
     </row>
     <row r="71" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="233" t="s">
-        <v>124</v>
-      </c>
+      <c r="A71" s="233"/>
       <c r="B71" s="359"/>
-      <c r="C71" s="359" t="s">
-        <v>109</v>
-      </c>
+      <c r="C71" s="359"/>
       <c r="D71" s="186"/>
       <c r="E71" s="336"/>
-      <c r="F71" s="360">
-        <v>-23</v>
-      </c>
-      <c r="G71" s="360">
-        <v>-28.4</v>
-      </c>
-      <c r="H71" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I71" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F71" s="360"/>
+      <c r="G71" s="360"/>
+      <c r="H71" s="348"/>
+      <c r="I71" s="233"/>
       <c r="J71" s="41"/>
       <c r="K71" s="41"/>
       <c r="L71" s="41"/>
@@ -7812,27 +7757,15 @@
       <c r="Y71" s="41"/>
     </row>
     <row r="72" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="233" t="s">
-        <v>125</v>
-      </c>
+      <c r="A72" s="233"/>
       <c r="B72" s="359"/>
-      <c r="C72" s="359" t="s">
-        <v>109</v>
-      </c>
+      <c r="C72" s="359"/>
       <c r="D72" s="186"/>
       <c r="E72" s="336"/>
-      <c r="F72" s="360">
-        <v>-18</v>
-      </c>
-      <c r="G72" s="360">
-        <v>-24.1</v>
-      </c>
-      <c r="H72" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I72" s="233" t="s">
-        <v>115</v>
-      </c>
+      <c r="F72" s="360"/>
+      <c r="G72" s="360"/>
+      <c r="H72" s="348"/>
+      <c r="I72" s="233"/>
       <c r="J72" s="41"/>
       <c r="K72" s="41"/>
       <c r="L72" s="41"/>
@@ -7851,27 +7784,15 @@
       <c r="Y72" s="41"/>
     </row>
     <row r="73" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="233" t="s">
-        <v>126</v>
-      </c>
+      <c r="A73" s="233"/>
       <c r="B73" s="346"/>
-      <c r="C73" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C73" s="346"/>
       <c r="D73" s="186"/>
       <c r="E73" s="336"/>
-      <c r="F73" s="347">
-        <v>-25</v>
-      </c>
-      <c r="G73" s="347">
-        <v>-26.1</v>
-      </c>
-      <c r="H73" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I73" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F73" s="347"/>
+      <c r="G73" s="347"/>
+      <c r="H73" s="348"/>
+      <c r="I73" s="233"/>
       <c r="J73" s="41"/>
       <c r="K73" s="41"/>
       <c r="L73" s="41"/>
@@ -7890,27 +7811,15 @@
       <c r="Y73" s="41"/>
     </row>
     <row r="74" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="299" t="s">
-        <v>127</v>
-      </c>
+      <c r="A74" s="299"/>
       <c r="B74" s="350"/>
-      <c r="C74" s="350" t="s">
-        <v>109</v>
-      </c>
+      <c r="C74" s="350"/>
       <c r="D74" s="299"/>
       <c r="E74" s="299"/>
-      <c r="F74" s="351">
-        <v>-2.5</v>
-      </c>
-      <c r="G74" s="351">
-        <v>-2.6</v>
-      </c>
-      <c r="H74" s="352" t="s">
-        <v>113</v>
-      </c>
-      <c r="I74" s="299" t="s">
-        <v>111</v>
-      </c>
+      <c r="F74" s="351"/>
+      <c r="G74" s="351"/>
+      <c r="H74" s="352"/>
+      <c r="I74" s="299"/>
       <c r="J74" s="41"/>
       <c r="K74" s="41"/>
       <c r="L74" s="41"/>
@@ -7929,27 +7838,15 @@
       <c r="Y74" s="41"/>
     </row>
     <row r="75" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="54" t="s">
-        <v>128</v>
-      </c>
+      <c r="A75" s="54"/>
       <c r="B75" s="342"/>
-      <c r="C75" s="342" t="s">
-        <v>109</v>
-      </c>
+      <c r="C75" s="342"/>
       <c r="D75" s="185"/>
       <c r="E75" s="57"/>
-      <c r="F75" s="353">
-        <v>-18</v>
-      </c>
-      <c r="G75" s="353">
-        <v>-17</v>
-      </c>
-      <c r="H75" s="344" t="s">
-        <v>113</v>
-      </c>
-      <c r="I75" s="54" t="s">
-        <v>111</v>
-      </c>
+      <c r="F75" s="353"/>
+      <c r="G75" s="353"/>
+      <c r="H75" s="344"/>
+      <c r="I75" s="54"/>
       <c r="J75" s="41"/>
       <c r="K75" s="41"/>
       <c r="L75" s="41"/>
@@ -7968,27 +7865,15 @@
       <c r="Y75" s="41"/>
     </row>
     <row r="76" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="233" t="s">
-        <v>129</v>
-      </c>
+      <c r="A76" s="233"/>
       <c r="B76" s="346"/>
-      <c r="C76" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C76" s="346"/>
       <c r="D76" s="226"/>
       <c r="E76" s="177"/>
-      <c r="F76" s="354">
-        <v>-2.5</v>
-      </c>
-      <c r="G76" s="354">
-        <v>-2.6</v>
-      </c>
-      <c r="H76" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I76" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F76" s="354"/>
+      <c r="G76" s="354"/>
+      <c r="H76" s="348"/>
+      <c r="I76" s="233"/>
       <c r="J76" s="41"/>
       <c r="K76" s="41"/>
       <c r="L76" s="41"/>
@@ -8007,27 +7892,15 @@
       <c r="Y76" s="41"/>
     </row>
     <row r="77" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="233" t="s">
-        <v>130</v>
-      </c>
+      <c r="A77" s="233"/>
       <c r="B77" s="346"/>
-      <c r="C77" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C77" s="346"/>
       <c r="D77" s="226"/>
       <c r="E77" s="177"/>
-      <c r="F77" s="347">
-        <v>-2.5</v>
-      </c>
-      <c r="G77" s="347">
-        <v>-2.5</v>
-      </c>
-      <c r="H77" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I77" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F77" s="347"/>
+      <c r="G77" s="347"/>
+      <c r="H77" s="348"/>
+      <c r="I77" s="233"/>
       <c r="J77" s="41"/>
       <c r="K77" s="41"/>
       <c r="L77" s="41"/>
@@ -8046,27 +7919,15 @@
       <c r="Y77" s="41"/>
     </row>
     <row r="78" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="233" t="s">
-        <v>131</v>
-      </c>
+      <c r="A78" s="233"/>
       <c r="B78" s="346"/>
-      <c r="C78" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C78" s="346"/>
       <c r="D78" s="226"/>
       <c r="E78" s="177"/>
-      <c r="F78" s="347">
-        <v>-25</v>
-      </c>
-      <c r="G78" s="347">
-        <v>-27.1</v>
-      </c>
-      <c r="H78" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I78" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F78" s="347"/>
+      <c r="G78" s="347"/>
+      <c r="H78" s="348"/>
+      <c r="I78" s="233"/>
       <c r="J78" s="41"/>
       <c r="K78" s="41"/>
       <c r="L78" s="41"/>
@@ -8085,27 +7946,15 @@
       <c r="Y78" s="41"/>
     </row>
     <row r="79" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="299" t="s">
-        <v>132</v>
-      </c>
+      <c r="A79" s="299"/>
       <c r="B79" s="350"/>
-      <c r="C79" s="350" t="s">
-        <v>109</v>
-      </c>
+      <c r="C79" s="350"/>
       <c r="D79" s="172"/>
       <c r="E79" s="173"/>
-      <c r="F79" s="351">
-        <v>0</v>
-      </c>
-      <c r="G79" s="351">
-        <v>0.1</v>
-      </c>
-      <c r="H79" s="352" t="s">
-        <v>113</v>
-      </c>
-      <c r="I79" s="299" t="s">
-        <v>115</v>
-      </c>
+      <c r="F79" s="351"/>
+      <c r="G79" s="351"/>
+      <c r="H79" s="352"/>
+      <c r="I79" s="299"/>
       <c r="J79" s="41"/>
       <c r="K79" s="41"/>
       <c r="L79" s="41"/>
@@ -8124,27 +7973,15 @@
       <c r="Y79" s="41"/>
     </row>
     <row r="80" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="54" t="s">
-        <v>133</v>
-      </c>
+      <c r="A80" s="54"/>
       <c r="B80" s="342"/>
-      <c r="C80" s="342" t="s">
-        <v>109</v>
-      </c>
+      <c r="C80" s="342"/>
       <c r="D80" s="185"/>
       <c r="E80" s="57"/>
-      <c r="F80" s="353">
-        <v>-18</v>
-      </c>
-      <c r="G80" s="353">
-        <v>-29.7</v>
-      </c>
-      <c r="H80" s="344" t="s">
-        <v>113</v>
-      </c>
-      <c r="I80" s="54" t="s">
-        <v>115</v>
-      </c>
+      <c r="F80" s="353"/>
+      <c r="G80" s="353"/>
+      <c r="H80" s="344"/>
+      <c r="I80" s="54"/>
       <c r="J80" s="41"/>
       <c r="K80" s="41"/>
       <c r="L80" s="41"/>
@@ -8163,27 +8000,15 @@
       <c r="Y80" s="41"/>
     </row>
     <row r="81" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="233" t="s">
-        <v>134</v>
-      </c>
+      <c r="A81" s="233"/>
       <c r="B81" s="346"/>
-      <c r="C81" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C81" s="346"/>
       <c r="D81" s="226"/>
       <c r="E81" s="177"/>
-      <c r="F81" s="354">
-        <v>-18</v>
-      </c>
-      <c r="G81" s="354">
-        <v>-17.7</v>
-      </c>
-      <c r="H81" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I81" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F81" s="354"/>
+      <c r="G81" s="354"/>
+      <c r="H81" s="348"/>
+      <c r="I81" s="233"/>
       <c r="J81" s="41"/>
       <c r="K81" s="41"/>
       <c r="L81" s="41"/>
@@ -8202,27 +8027,15 @@
       <c r="Y81" s="41"/>
     </row>
     <row r="82" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="233" t="s">
-        <v>135</v>
-      </c>
+      <c r="A82" s="233"/>
       <c r="B82" s="346"/>
-      <c r="C82" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C82" s="346"/>
       <c r="D82" s="226"/>
       <c r="E82" s="177"/>
-      <c r="F82" s="354">
-        <v>-23</v>
-      </c>
-      <c r="G82" s="354">
-        <v>-27.3</v>
-      </c>
-      <c r="H82" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I82" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F82" s="354"/>
+      <c r="G82" s="354"/>
+      <c r="H82" s="348"/>
+      <c r="I82" s="233"/>
       <c r="J82" s="41"/>
       <c r="K82" s="41"/>
       <c r="L82" s="41"/>
@@ -8241,27 +8054,15 @@
       <c r="Y82" s="41"/>
     </row>
     <row r="83" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="233" t="s">
-        <v>136</v>
-      </c>
+      <c r="A83" s="233"/>
       <c r="B83" s="346"/>
-      <c r="C83" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C83" s="346"/>
       <c r="D83" s="226"/>
       <c r="E83" s="177"/>
-      <c r="F83" s="354">
-        <v>-2.6</v>
-      </c>
-      <c r="G83" s="354">
-        <v>-2.5</v>
-      </c>
-      <c r="H83" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I83" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F83" s="354"/>
+      <c r="G83" s="354"/>
+      <c r="H83" s="348"/>
+      <c r="I83" s="233"/>
       <c r="J83" s="41"/>
       <c r="K83" s="41"/>
       <c r="L83" s="41"/>
@@ -8280,27 +8081,15 @@
       <c r="Y83" s="41"/>
     </row>
     <row r="84" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="233" t="s">
-        <v>137</v>
-      </c>
+      <c r="A84" s="233"/>
       <c r="B84" s="346"/>
-      <c r="C84" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C84" s="346"/>
       <c r="D84" s="226"/>
       <c r="E84" s="177"/>
-      <c r="F84" s="347">
-        <v>-2.5</v>
-      </c>
-      <c r="G84" s="347">
-        <v>-2.5</v>
-      </c>
-      <c r="H84" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I84" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F84" s="347"/>
+      <c r="G84" s="347"/>
+      <c r="H84" s="348"/>
+      <c r="I84" s="233"/>
       <c r="J84" s="41"/>
       <c r="K84" s="41"/>
       <c r="L84" s="41"/>
@@ -8868,14 +8657,14 @@
       <c r="D104" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E104" s="206" t="s">
+      <c r="E104" s="208" t="s">
         <v>145</v>
       </c>
       <c r="F104" s="206"/>
       <c r="G104" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="H104" s="207">
+      <c r="H104" s="560">
         <v>46229</v>
       </c>
       <c r="I104" s="8"/>
@@ -8905,14 +8694,14 @@
       <c r="D105" s="334" t="s">
         <v>7</v>
       </c>
-      <c r="E105" s="8">
+      <c r="E105" s="208">
         <v>16</v>
       </c>
       <c r="F105" s="3"/>
       <c r="G105" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="H105" s="8" t="s">
+      <c r="H105" s="208" t="s">
         <v>95</v>
       </c>
       <c r="I105" s="8"/>
@@ -9037,27 +8826,17 @@
       <c r="Y108" s="105"/>
     </row>
     <row r="109" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="54" t="s">
-        <v>146</v>
-      </c>
+      <c r="A109" s="54"/>
       <c r="B109" s="342"/>
-      <c r="C109" s="342" t="s">
-        <v>109</v>
-      </c>
+      <c r="C109" s="342"/>
       <c r="D109" s="185"/>
       <c r="E109" s="57"/>
-      <c r="F109" s="343">
-        <v>-2.5</v>
-      </c>
-      <c r="G109" s="343">
-        <v>-2.5</v>
-      </c>
+      <c r="F109" s="343"/>
+      <c r="G109" s="343"/>
       <c r="H109" s="344" t="s">
         <v>110</v>
       </c>
-      <c r="I109" s="54" t="s">
-        <v>111</v>
-      </c>
+      <c r="I109" s="54"/>
       <c r="J109" s="41"/>
       <c r="K109" s="41"/>
       <c r="L109" s="41"/>
@@ -9076,27 +8855,15 @@
       <c r="Y109" s="41"/>
     </row>
     <row r="110" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="233" t="s">
-        <v>147</v>
-      </c>
+      <c r="A110" s="233"/>
       <c r="B110" s="346"/>
-      <c r="C110" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C110" s="346"/>
       <c r="D110" s="226"/>
       <c r="E110" s="177"/>
-      <c r="F110" s="347">
-        <v>-2.6</v>
-      </c>
-      <c r="G110" s="347">
-        <v>-2.6</v>
-      </c>
-      <c r="H110" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I110" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F110" s="347"/>
+      <c r="G110" s="347"/>
+      <c r="H110" s="348"/>
+      <c r="I110" s="233"/>
       <c r="J110" s="41"/>
       <c r="K110" s="41"/>
       <c r="L110" s="41"/>
@@ -9115,27 +8882,15 @@
       <c r="Y110" s="41"/>
     </row>
     <row r="111" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="233" t="s">
-        <v>148</v>
-      </c>
+      <c r="A111" s="233"/>
       <c r="B111" s="346"/>
-      <c r="C111" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C111" s="346"/>
       <c r="D111" s="226"/>
       <c r="E111" s="177"/>
-      <c r="F111" s="347">
-        <v>-18</v>
-      </c>
-      <c r="G111" s="347">
-        <v>-22.5</v>
-      </c>
-      <c r="H111" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I111" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F111" s="347"/>
+      <c r="G111" s="347"/>
+      <c r="H111" s="348"/>
+      <c r="I111" s="233"/>
       <c r="J111" s="41"/>
       <c r="K111" s="41"/>
       <c r="L111" s="41"/>
@@ -9154,27 +8909,15 @@
       <c r="Y111" s="41"/>
     </row>
     <row r="112" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A112" s="233" t="s">
-        <v>149</v>
-      </c>
+      <c r="A112" s="233"/>
       <c r="B112" s="346"/>
-      <c r="C112" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C112" s="346"/>
       <c r="D112" s="226"/>
       <c r="E112" s="177"/>
-      <c r="F112" s="347">
-        <v>-18</v>
-      </c>
-      <c r="G112" s="347">
-        <v>-18</v>
-      </c>
-      <c r="H112" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I112" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F112" s="347"/>
+      <c r="G112" s="347"/>
+      <c r="H112" s="348"/>
+      <c r="I112" s="233"/>
       <c r="J112" s="41"/>
       <c r="K112" s="41"/>
       <c r="L112" s="41"/>
@@ -9193,27 +8936,15 @@
       <c r="Y112" s="41"/>
     </row>
     <row r="113" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="299" t="s">
-        <v>150</v>
-      </c>
+      <c r="A113" s="299"/>
       <c r="B113" s="350"/>
-      <c r="C113" s="350" t="s">
-        <v>109</v>
-      </c>
+      <c r="C113" s="350"/>
       <c r="D113" s="172"/>
       <c r="E113" s="173"/>
-      <c r="F113" s="351">
-        <v>-18</v>
-      </c>
-      <c r="G113" s="351">
-        <v>-22.9</v>
-      </c>
-      <c r="H113" s="352" t="s">
-        <v>113</v>
-      </c>
-      <c r="I113" s="299" t="s">
-        <v>115</v>
-      </c>
+      <c r="F113" s="351"/>
+      <c r="G113" s="351"/>
+      <c r="H113" s="352"/>
+      <c r="I113" s="299"/>
       <c r="J113" s="41"/>
       <c r="K113" s="41"/>
       <c r="L113" s="41"/>
@@ -9232,27 +8963,15 @@
       <c r="Y113" s="41"/>
     </row>
     <row r="114" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="54" t="s">
-        <v>151</v>
-      </c>
+      <c r="A114" s="54"/>
       <c r="B114" s="342"/>
-      <c r="C114" s="342" t="s">
-        <v>109</v>
-      </c>
+      <c r="C114" s="342"/>
       <c r="D114" s="185"/>
       <c r="E114" s="57"/>
-      <c r="F114" s="353">
-        <v>-18</v>
-      </c>
-      <c r="G114" s="353">
-        <v>-23.9</v>
-      </c>
-      <c r="H114" s="344" t="s">
-        <v>113</v>
-      </c>
-      <c r="I114" s="54" t="s">
-        <v>111</v>
-      </c>
+      <c r="F114" s="353"/>
+      <c r="G114" s="353"/>
+      <c r="H114" s="344"/>
+      <c r="I114" s="54"/>
       <c r="J114" s="41"/>
       <c r="K114" s="41"/>
       <c r="L114" s="41"/>
@@ -9271,27 +8990,15 @@
       <c r="Y114" s="41"/>
     </row>
     <row r="115" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="233" t="s">
-        <v>152</v>
-      </c>
+      <c r="A115" s="233"/>
       <c r="B115" s="346"/>
-      <c r="C115" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C115" s="346"/>
       <c r="D115" s="226"/>
       <c r="E115" s="177"/>
-      <c r="F115" s="354">
-        <v>-18</v>
-      </c>
-      <c r="G115" s="354">
-        <v>-22.8</v>
-      </c>
-      <c r="H115" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I115" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F115" s="354"/>
+      <c r="G115" s="354"/>
+      <c r="H115" s="348"/>
+      <c r="I115" s="233"/>
       <c r="J115" s="41"/>
       <c r="K115" s="41"/>
       <c r="L115" s="41"/>
@@ -9310,27 +9017,15 @@
       <c r="Y115" s="41"/>
     </row>
     <row r="116" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="233" t="s">
-        <v>153</v>
-      </c>
+      <c r="A116" s="233"/>
       <c r="B116" s="346"/>
-      <c r="C116" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C116" s="346"/>
       <c r="D116" s="226"/>
       <c r="E116" s="177"/>
-      <c r="F116" s="347">
-        <v>-18</v>
-      </c>
-      <c r="G116" s="347">
-        <v>-23.8</v>
-      </c>
-      <c r="H116" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I116" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F116" s="347"/>
+      <c r="G116" s="347"/>
+      <c r="H116" s="348"/>
+      <c r="I116" s="233"/>
       <c r="J116" s="41"/>
       <c r="K116" s="41"/>
       <c r="L116" s="41"/>
@@ -9349,27 +9044,15 @@
       <c r="Y116" s="41"/>
     </row>
     <row r="117" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="233" t="s">
-        <v>154</v>
-      </c>
+      <c r="A117" s="233"/>
       <c r="B117" s="346"/>
-      <c r="C117" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C117" s="346"/>
       <c r="D117" s="226"/>
       <c r="E117" s="177"/>
-      <c r="F117" s="354">
-        <v>-2</v>
-      </c>
-      <c r="G117" s="347">
-        <v>-2</v>
-      </c>
-      <c r="H117" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I117" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F117" s="354"/>
+      <c r="G117" s="347"/>
+      <c r="H117" s="348"/>
+      <c r="I117" s="233"/>
       <c r="J117" s="41"/>
       <c r="K117" s="41"/>
       <c r="L117" s="41"/>
@@ -9388,27 +9071,15 @@
       <c r="Y117" s="41"/>
     </row>
     <row r="118" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="299" t="s">
-        <v>155</v>
-      </c>
+      <c r="A118" s="299"/>
       <c r="B118" s="350"/>
-      <c r="C118" s="350" t="s">
-        <v>109</v>
-      </c>
+      <c r="C118" s="350"/>
       <c r="D118" s="172"/>
       <c r="E118" s="173"/>
-      <c r="F118" s="351">
-        <v>-18</v>
-      </c>
-      <c r="G118" s="351">
-        <v>-26.6</v>
-      </c>
-      <c r="H118" s="352" t="s">
-        <v>113</v>
-      </c>
-      <c r="I118" s="299" t="s">
-        <v>111</v>
-      </c>
+      <c r="F118" s="351"/>
+      <c r="G118" s="351"/>
+      <c r="H118" s="352"/>
+      <c r="I118" s="299"/>
       <c r="J118" s="41"/>
       <c r="K118" s="41"/>
       <c r="L118" s="41"/>
@@ -9427,27 +9098,15 @@
       <c r="Y118" s="41"/>
     </row>
     <row r="119" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="54" t="s">
-        <v>156</v>
-      </c>
+      <c r="A119" s="54"/>
       <c r="B119" s="342"/>
-      <c r="C119" s="342" t="s">
-        <v>109</v>
-      </c>
+      <c r="C119" s="342"/>
       <c r="D119" s="252"/>
       <c r="E119" s="253"/>
-      <c r="F119" s="355">
-        <v>-2.5</v>
-      </c>
-      <c r="G119" s="355">
-        <v>-2.5</v>
-      </c>
-      <c r="H119" s="344" t="s">
-        <v>113</v>
-      </c>
-      <c r="I119" s="54" t="s">
-        <v>111</v>
-      </c>
+      <c r="F119" s="355"/>
+      <c r="G119" s="355"/>
+      <c r="H119" s="344"/>
+      <c r="I119" s="54"/>
       <c r="J119" s="41"/>
       <c r="K119" s="41"/>
       <c r="L119" s="41"/>
@@ -9466,27 +9125,15 @@
       <c r="Y119" s="41"/>
     </row>
     <row r="120" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="233" t="s">
-        <v>157</v>
-      </c>
+      <c r="A120" s="233"/>
       <c r="B120" s="346"/>
-      <c r="C120" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C120" s="346"/>
       <c r="D120" s="186"/>
       <c r="E120" s="336"/>
-      <c r="F120" s="347">
-        <v>-2</v>
-      </c>
-      <c r="G120" s="347">
-        <v>-2.1</v>
-      </c>
-      <c r="H120" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I120" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F120" s="347"/>
+      <c r="G120" s="347"/>
+      <c r="H120" s="348"/>
+      <c r="I120" s="233"/>
       <c r="J120" s="41"/>
       <c r="K120" s="41"/>
       <c r="L120" s="41"/>
@@ -9505,27 +9152,15 @@
       <c r="Y120" s="41"/>
     </row>
     <row r="121" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A121" s="233" t="s">
-        <v>158</v>
-      </c>
+      <c r="A121" s="233"/>
       <c r="B121" s="346"/>
-      <c r="C121" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C121" s="346"/>
       <c r="D121" s="186"/>
       <c r="E121" s="336"/>
-      <c r="F121" s="347">
-        <v>-2.5</v>
-      </c>
-      <c r="G121" s="347">
-        <v>-2.5</v>
-      </c>
-      <c r="H121" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I121" s="233" t="s">
-        <v>111</v>
-      </c>
+      <c r="F121" s="347"/>
+      <c r="G121" s="347"/>
+      <c r="H121" s="348"/>
+      <c r="I121" s="233"/>
       <c r="J121" s="41"/>
       <c r="K121" s="41"/>
       <c r="L121" s="41"/>
@@ -9544,27 +9179,15 @@
       <c r="Y121" s="41"/>
     </row>
     <row r="122" ht="16.9" customHeight="1" spans="1:25" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="233" t="s">
-        <v>159</v>
-      </c>
+      <c r="A122" s="233"/>
       <c r="B122" s="346"/>
-      <c r="C122" s="346" t="s">
-        <v>109</v>
-      </c>
+      <c r="C122" s="346"/>
       <c r="D122" s="186"/>
       <c r="E122" s="336"/>
-      <c r="F122" s="347">
-        <v>-18</v>
-      </c>
-      <c r="G122" s="347">
-        <v>-13</v>
-      </c>
-      <c r="H122" s="348" t="s">
-        <v>113</v>
-      </c>
-      <c r="I122" s="233" t="s">
-        <v>115</v>
-      </c>
+      <c r="F122" s="347"/>
+      <c r="G122" s="347"/>
+      <c r="H122" s="348"/>
+      <c r="I122" s="233"/>
       <c r="J122" s="41"/>
       <c r="K122" s="41"/>
       <c r="L122" s="41"/>
@@ -10210,7 +9833,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor indexed="59"/>
   </sheetPr>
@@ -10505,7 +10128,7 @@
       <c r="X1" s="3"/>
       <c r="Y1" s="3"/>
     </row>
-    <row r="2" ht="21.75" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="2" ht="24.3" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>1</v>
@@ -10565,7 +10188,7 @@
       <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="544" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="1"/>
@@ -10574,14 +10197,14 @@
       <c r="F4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="12"/>
+      <c r="G4" s="545"/>
       <c r="H4" s="12"/>
       <c r="I4" s="12"/>
       <c r="J4" s="1"/>
       <c r="K4" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="L4" s="14"/>
+      <c r="L4" s="546"/>
       <c r="M4" s="15"/>
       <c r="N4" s="15"/>
       <c r="O4" s="15"/>
@@ -10627,21 +10250,21 @@
       <c r="A6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="17"/>
+      <c r="B6" s="545"/>
       <c r="C6" s="1"/>
       <c r="D6" s="2"/>
       <c r="E6" s="18"/>
       <c r="F6" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="12"/>
+      <c r="G6" s="545"/>
       <c r="H6" s="12"/>
       <c r="I6" s="12"/>
       <c r="J6" s="1"/>
       <c r="K6" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="L6" s="19" t="s">
+      <c r="L6" s="547" t="s">
         <v>9</v>
       </c>
       <c r="M6" s="19"/>
@@ -13235,7 +12858,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="1" tint="0.499984740745262"/>
   </sheetPr>
@@ -13896,7 +13519,7 @@
       </c>
       <c r="B6" s="258"/>
       <c r="C6" s="258"/>
-      <c r="D6" s="258" t="s">
+      <c r="D6" s="535" t="s">
         <v>38</v>
       </c>
       <c r="E6" s="258"/>
@@ -13912,7 +13535,7 @@
       <c r="O6" s="258" t="s">
         <v>4</v>
       </c>
-      <c r="P6" s="41"/>
+      <c r="P6" s="570"/>
       <c r="Q6" s="41"/>
       <c r="R6" s="105" t="s">
         <v>163</v>
@@ -13928,7 +13551,7 @@
       </c>
       <c r="Z6" s="105"/>
       <c r="AA6" s="105"/>
-      <c r="AB6" s="365">
+      <c r="AB6" s="571">
         <v>46229</v>
       </c>
       <c r="AC6" s="366"/>
@@ -13984,7 +13607,7 @@
       </c>
       <c r="B8" s="367"/>
       <c r="C8" s="367"/>
-      <c r="D8" s="368" t="s">
+      <c r="D8" s="572" t="s">
         <v>65</v>
       </c>
       <c r="E8" s="368"/>
@@ -14000,7 +13623,7 @@
       <c r="O8" s="368" t="s">
         <v>7</v>
       </c>
-      <c r="P8" s="369"/>
+      <c r="P8" s="572"/>
       <c r="Q8" s="369"/>
       <c r="R8" s="367">
         <v>16</v>
@@ -14016,7 +13639,7 @@
       </c>
       <c r="Z8" s="367"/>
       <c r="AA8" s="367"/>
-      <c r="AB8" s="367" t="s">
+      <c r="AB8" s="572" t="s">
         <v>25</v>
       </c>
       <c r="AC8" s="367"/>
@@ -18671,7 +18294,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor indexed="60"/>
   </sheetPr>
@@ -19464,7 +19087,7 @@
       <c r="A6" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="206" t="s">
+      <c r="B6" s="208" t="s">
         <v>38</v>
       </c>
       <c r="C6" s="3"/>
@@ -19474,13 +19097,13 @@
       <c r="G6" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="H6" s="8"/>
+      <c r="H6" s="208"/>
       <c r="I6" s="8"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="L6" s="207"/>
+      <c r="L6" s="560"/>
       <c r="M6" s="8"/>
       <c r="N6" s="1"/>
       <c r="O6" s="3"/>
@@ -19526,7 +19149,7 @@
       <c r="A8" s="206" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="561" t="s">
         <v>25</v>
       </c>
       <c r="C8" s="3"/>
@@ -19536,13 +19159,13 @@
       <c r="G8" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="H8" s="8"/>
+      <c r="H8" s="208"/>
       <c r="I8" s="8"/>
       <c r="J8" s="3"/>
       <c r="K8" s="206" t="s">
         <v>43</v>
       </c>
-      <c r="L8" s="8"/>
+      <c r="L8" s="208"/>
       <c r="M8" s="8"/>
       <c r="N8" s="3"/>
       <c r="O8" s="3"/>
@@ -19584,7 +19207,7 @@
       <c r="X9" s="3"/>
       <c r="Y9" s="3"/>
     </row>
-    <row r="10" ht="14.45" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="10" ht="16.2" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="209" t="s">
         <v>44</v>
       </c>
@@ -19629,7 +19252,7 @@
       <c r="X10" s="3"/>
       <c r="Y10" s="3"/>
     </row>
-    <row r="11" ht="14.45" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="11" ht="16.2" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="213"/>
       <c r="B11" s="214"/>
       <c r="C11" s="215"/>
@@ -19663,15 +19286,15 @@
       <c r="B12" s="218"/>
       <c r="C12" s="219"/>
       <c r="D12" s="218"/>
-      <c r="E12" s="220"/>
-      <c r="F12" s="221"/>
+      <c r="E12" s="267"/>
+      <c r="F12" s="219"/>
       <c r="G12" s="217"/>
       <c r="H12" s="222"/>
       <c r="I12" s="223"/>
       <c r="J12" s="224"/>
       <c r="K12" s="217"/>
       <c r="L12" s="217"/>
-      <c r="M12" s="225"/>
+      <c r="M12" s="562"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
@@ -19690,15 +19313,15 @@
       <c r="B13" s="226"/>
       <c r="C13" s="177"/>
       <c r="D13" s="185"/>
-      <c r="E13" s="227"/>
-      <c r="F13" s="228"/>
+      <c r="E13" s="55"/>
+      <c r="F13" s="57"/>
       <c r="G13" s="54"/>
       <c r="H13" s="229"/>
       <c r="I13" s="230"/>
       <c r="J13" s="231"/>
       <c r="K13" s="54"/>
       <c r="L13" s="54"/>
-      <c r="M13" s="232"/>
+      <c r="M13" s="563"/>
       <c r="N13" s="3"/>
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
@@ -19717,15 +19340,15 @@
       <c r="B14" s="226"/>
       <c r="C14" s="177"/>
       <c r="D14" s="226"/>
-      <c r="E14" s="234"/>
-      <c r="F14" s="235"/>
+      <c r="E14" s="272"/>
+      <c r="F14" s="177"/>
       <c r="G14" s="233"/>
       <c r="H14" s="236"/>
       <c r="I14" s="237"/>
       <c r="J14" s="236"/>
       <c r="K14" s="233"/>
       <c r="L14" s="233"/>
-      <c r="M14" s="238"/>
+      <c r="M14" s="564"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
@@ -19744,15 +19367,15 @@
       <c r="B15" s="185"/>
       <c r="C15" s="57"/>
       <c r="D15" s="185"/>
-      <c r="E15" s="227"/>
-      <c r="F15" s="228"/>
+      <c r="E15" s="55"/>
+      <c r="F15" s="57"/>
       <c r="G15" s="54"/>
       <c r="H15" s="239"/>
       <c r="I15" s="240"/>
       <c r="J15" s="231"/>
       <c r="K15" s="54"/>
       <c r="L15" s="54"/>
-      <c r="M15" s="232"/>
+      <c r="M15" s="563"/>
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
       <c r="P15" s="3"/>
@@ -19771,15 +19394,15 @@
       <c r="B16" s="226"/>
       <c r="C16" s="177"/>
       <c r="D16" s="185"/>
-      <c r="E16" s="227"/>
-      <c r="F16" s="228"/>
+      <c r="E16" s="55"/>
+      <c r="F16" s="57"/>
       <c r="G16" s="54"/>
       <c r="H16" s="229"/>
       <c r="I16" s="230"/>
       <c r="J16" s="231"/>
       <c r="K16" s="54"/>
       <c r="L16" s="54"/>
-      <c r="M16" s="232"/>
+      <c r="M16" s="563"/>
       <c r="N16" s="3"/>
       <c r="O16" s="3"/>
       <c r="P16" s="3"/>
@@ -19798,15 +19421,15 @@
       <c r="B17" s="226"/>
       <c r="C17" s="177"/>
       <c r="D17" s="226"/>
-      <c r="E17" s="234"/>
-      <c r="F17" s="235"/>
+      <c r="E17" s="272"/>
+      <c r="F17" s="177"/>
       <c r="G17" s="233"/>
       <c r="H17" s="236"/>
       <c r="I17" s="237"/>
       <c r="J17" s="236"/>
       <c r="K17" s="233"/>
       <c r="L17" s="233"/>
-      <c r="M17" s="238"/>
+      <c r="M17" s="564"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
@@ -20659,7 +20282,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor indexed="60"/>
   </sheetPr>
@@ -21388,7 +21011,7 @@
       <c r="A6" s="206" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="206" t="s">
+      <c r="B6" s="208" t="s">
         <v>38</v>
       </c>
       <c r="C6" s="3"/>
@@ -21400,7 +21023,7 @@
         <v>60</v>
       </c>
       <c r="I6" s="8"/>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="208" t="s">
         <v>61</v>
       </c>
       <c r="K6" s="8"/>
@@ -21410,7 +21033,7 @@
       <c r="O6" s="206" t="s">
         <v>62</v>
       </c>
-      <c r="P6" s="207">
+      <c r="P6" s="560">
         <v>46229</v>
       </c>
       <c r="Q6" s="8"/>
@@ -21454,7 +21077,7 @@
       <c r="A8" s="206" t="s">
         <v>63</v>
       </c>
-      <c r="B8" s="206" t="s">
+      <c r="B8" s="208" t="s">
         <v>25</v>
       </c>
       <c r="C8" s="206"/>
@@ -21466,7 +21089,7 @@
         <v>64</v>
       </c>
       <c r="I8" s="8"/>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="208" t="s">
         <v>65</v>
       </c>
       <c r="K8" s="8"/>
@@ -21476,7 +21099,7 @@
       <c r="O8" s="206" t="s">
         <v>66</v>
       </c>
-      <c r="P8" s="8">
+      <c r="P8" s="208">
         <v>16</v>
       </c>
       <c r="Q8" s="8"/>
@@ -21516,7 +21139,7 @@
       <c r="X9" s="3"/>
       <c r="Y9" s="3"/>
     </row>
-    <row r="10" ht="12" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="10" ht="16.2" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="209" t="s">
         <v>11</v>
       </c>
@@ -21557,7 +21180,7 @@
       <c r="X10" s="3"/>
       <c r="Y10" s="3"/>
     </row>
-    <row r="11" ht="12" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="11" ht="16.2" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="213"/>
       <c r="B11" s="213"/>
       <c r="C11" s="264"/>
@@ -22371,7 +21994,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Y47"/>
   <sheetFormatPr defaultRowHeight="17.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
@@ -23037,17 +22660,17 @@
       <c r="A6" s="156" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="157"/>
+      <c r="B6" s="548"/>
       <c r="C6" s="156" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="15"/>
+      <c r="D6" s="549"/>
       <c r="E6" s="15"/>
       <c r="F6" s="9"/>
       <c r="G6" s="158" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="159">
+      <c r="H6" s="550">
         <v>46229</v>
       </c>
       <c r="I6" s="9"/>
@@ -23099,17 +22722,17 @@
       <c r="A8" s="156" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="160"/>
+      <c r="B8" s="549"/>
       <c r="C8" s="156" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="15"/>
+      <c r="D8" s="549"/>
       <c r="E8" s="15"/>
       <c r="F8" s="156"/>
       <c r="G8" s="161" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="19"/>
+      <c r="H8" s="547"/>
       <c r="I8" s="9"/>
       <c r="J8" s="9"/>
       <c r="K8" s="9"/>
@@ -23247,7 +22870,7 @@
         <v>34</v>
       </c>
       <c r="B13" s="166"/>
-      <c r="C13" s="167"/>
+      <c r="C13" s="217"/>
       <c r="D13" s="167"/>
       <c r="E13" s="167"/>
       <c r="F13" s="167"/>
@@ -23274,7 +22897,7 @@
     <row r="14" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="168"/>
       <c r="B14" s="169"/>
-      <c r="C14" s="170"/>
+      <c r="C14" s="233"/>
       <c r="D14" s="170"/>
       <c r="E14" s="170"/>
       <c r="F14" s="170"/>
@@ -23301,7 +22924,7 @@
     <row r="15" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="168"/>
       <c r="B15" s="57"/>
-      <c r="C15" s="171"/>
+      <c r="C15" s="54"/>
       <c r="D15" s="171"/>
       <c r="E15" s="171"/>
       <c r="F15" s="171"/>
@@ -23328,7 +22951,7 @@
     <row r="16" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="168"/>
       <c r="B16" s="57"/>
-      <c r="C16" s="171"/>
+      <c r="C16" s="54"/>
       <c r="D16" s="171"/>
       <c r="E16" s="171"/>
       <c r="F16" s="171"/>
@@ -23355,7 +22978,7 @@
     <row r="17" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" s="172"/>
       <c r="B17" s="173"/>
-      <c r="C17" s="174"/>
+      <c r="C17" s="299"/>
       <c r="D17" s="174"/>
       <c r="E17" s="174"/>
       <c r="F17" s="174"/>
@@ -23384,7 +23007,7 @@
     <row r="18" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" s="175"/>
       <c r="B18" s="57"/>
-      <c r="C18" s="171"/>
+      <c r="C18" s="54"/>
       <c r="D18" s="171"/>
       <c r="E18" s="171"/>
       <c r="F18" s="171"/>
@@ -23411,7 +23034,7 @@
     <row r="19" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" s="176"/>
       <c r="B19" s="57"/>
-      <c r="C19" s="171"/>
+      <c r="C19" s="54"/>
       <c r="D19" s="171"/>
       <c r="E19" s="171"/>
       <c r="F19" s="171"/>
@@ -23438,7 +23061,7 @@
     <row r="20" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" s="168"/>
       <c r="B20" s="177"/>
-      <c r="C20" s="170"/>
+      <c r="C20" s="233"/>
       <c r="D20" s="170"/>
       <c r="E20" s="170"/>
       <c r="F20" s="170"/>
@@ -23465,7 +23088,7 @@
     <row r="21" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" s="168"/>
       <c r="B21" s="178"/>
-      <c r="C21" s="179"/>
+      <c r="C21" s="551"/>
       <c r="D21" s="179"/>
       <c r="E21" s="179"/>
       <c r="F21" s="179"/>
@@ -23494,7 +23117,7 @@
     <row r="22" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" s="180"/>
       <c r="B22" s="177"/>
-      <c r="C22" s="181"/>
+      <c r="C22" s="552"/>
       <c r="D22" s="181"/>
       <c r="E22" s="181"/>
       <c r="F22" s="181"/>
@@ -23521,7 +23144,7 @@
     <row r="23" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" s="182"/>
       <c r="B23" s="102"/>
-      <c r="C23" s="183"/>
+      <c r="C23" s="553"/>
       <c r="D23" s="183"/>
       <c r="E23" s="183"/>
       <c r="F23" s="183"/>
@@ -23548,7 +23171,7 @@
     <row r="24" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A24" s="175"/>
       <c r="B24" s="57"/>
-      <c r="C24" s="184"/>
+      <c r="C24" s="554"/>
       <c r="D24" s="184"/>
       <c r="E24" s="184"/>
       <c r="F24" s="184"/>
@@ -23575,7 +23198,7 @@
     <row r="25" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25" s="185"/>
       <c r="B25" s="177"/>
-      <c r="C25" s="181"/>
+      <c r="C25" s="552"/>
       <c r="D25" s="181"/>
       <c r="E25" s="181"/>
       <c r="F25" s="181"/>
@@ -23602,7 +23225,7 @@
     <row r="26" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" s="186"/>
       <c r="B26" s="169"/>
-      <c r="C26" s="184"/>
+      <c r="C26" s="554"/>
       <c r="D26" s="184"/>
       <c r="E26" s="184"/>
       <c r="F26" s="184"/>
@@ -23629,7 +23252,7 @@
     <row r="27" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27" s="168"/>
       <c r="B27" s="57"/>
-      <c r="C27" s="184"/>
+      <c r="C27" s="554"/>
       <c r="D27" s="184"/>
       <c r="E27" s="184"/>
       <c r="F27" s="184"/>
@@ -23656,7 +23279,7 @@
     <row r="28" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28" s="187"/>
       <c r="B28" s="173"/>
-      <c r="C28" s="188"/>
+      <c r="C28" s="555"/>
       <c r="D28" s="189"/>
       <c r="E28" s="189"/>
       <c r="F28" s="189"/>
@@ -23683,7 +23306,7 @@
     <row r="29" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29" s="191"/>
       <c r="B29" s="28"/>
-      <c r="C29" s="192"/>
+      <c r="C29" s="556"/>
       <c r="D29" s="192"/>
       <c r="E29" s="192"/>
       <c r="F29" s="192"/>
@@ -23710,7 +23333,7 @@
     <row r="30" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" s="176"/>
       <c r="B30" s="57"/>
-      <c r="C30" s="193"/>
+      <c r="C30" s="557"/>
       <c r="D30" s="194"/>
       <c r="E30" s="194"/>
       <c r="F30" s="194"/>
@@ -23737,7 +23360,7 @@
     <row r="31" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31" s="185"/>
       <c r="B31" s="177"/>
-      <c r="C31" s="196"/>
+      <c r="C31" s="558"/>
       <c r="D31" s="197"/>
       <c r="E31" s="197"/>
       <c r="F31" s="197"/>
@@ -23764,7 +23387,7 @@
     <row r="32" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A32" s="186"/>
       <c r="B32" s="57"/>
-      <c r="C32" s="184"/>
+      <c r="C32" s="554"/>
       <c r="D32" s="184"/>
       <c r="E32" s="184"/>
       <c r="F32" s="184"/>
@@ -23791,7 +23414,7 @@
     <row r="33" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A33" s="172"/>
       <c r="B33" s="173"/>
-      <c r="C33" s="199"/>
+      <c r="C33" s="559"/>
       <c r="D33" s="199"/>
       <c r="E33" s="199"/>
       <c r="F33" s="199"/>
@@ -23818,7 +23441,7 @@
     <row r="34" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A34" s="200"/>
       <c r="B34" s="57"/>
-      <c r="C34" s="184"/>
+      <c r="C34" s="554"/>
       <c r="D34" s="184"/>
       <c r="E34" s="184"/>
       <c r="F34" s="184"/>
@@ -23845,7 +23468,7 @@
     <row r="35" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A35" s="201"/>
       <c r="B35" s="57"/>
-      <c r="C35" s="184"/>
+      <c r="C35" s="554"/>
       <c r="D35" s="184"/>
       <c r="E35" s="184"/>
       <c r="F35" s="184"/>
@@ -23872,7 +23495,7 @@
     <row r="36" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A36" s="201"/>
       <c r="B36" s="57"/>
-      <c r="C36" s="184"/>
+      <c r="C36" s="554"/>
       <c r="D36" s="184"/>
       <c r="E36" s="184"/>
       <c r="F36" s="184"/>
@@ -23899,7 +23522,7 @@
     <row r="37" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A37" s="168"/>
       <c r="B37" s="57"/>
-      <c r="C37" s="184"/>
+      <c r="C37" s="554"/>
       <c r="D37" s="184"/>
       <c r="E37" s="184"/>
       <c r="F37" s="184"/>
@@ -23926,7 +23549,7 @@
     <row r="38" ht="19.9" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A38" s="168"/>
       <c r="B38" s="57"/>
-      <c r="C38" s="184"/>
+      <c r="C38" s="554"/>
       <c r="D38" s="184"/>
       <c r="E38" s="184"/>
       <c r="F38" s="184"/>
@@ -24196,7 +23819,7 @@
       <c r="Y47" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="36">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="C3:F3"/>
@@ -24231,6 +23854,8 @@
     <mergeCell ref="C37:H37"/>
     <mergeCell ref="C38:H38"/>
     <mergeCell ref="A42:B42"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C40:H40"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.3937007874015748" right="0.3937007874015748" top="0.3937007874015748" bottom="0.3937007874015748" header="0.5118110236220472" footer="0.35433070866141736"/>
@@ -24239,7 +23864,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Y42"/>
   <sheetFormatPr defaultRowHeight="17.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
@@ -24909,7 +24534,7 @@
       <c r="A4" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B4" s="206" t="s">
+      <c r="B4" s="208" t="s">
         <v>38</v>
       </c>
       <c r="C4" s="206"/>
@@ -24918,7 +24543,7 @@
       <c r="F4" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="G4" s="207"/>
+      <c r="G4" s="560"/>
       <c r="H4" s="8"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
@@ -24969,7 +24594,7 @@
       <c r="A6" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="206" t="s">
+      <c r="B6" s="208" t="s">
         <v>61</v>
       </c>
       <c r="C6" s="206"/>
@@ -24980,7 +24605,7 @@
       <c r="F6" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="G6" s="275" t="s">
+      <c r="G6" s="565" t="s">
         <v>25</v>
       </c>
       <c r="H6" s="3"/>
@@ -25625,12 +25250,12 @@
     <row r="29" ht="23.1" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29" s="322"/>
       <c r="B29" s="323"/>
-      <c r="C29" s="324"/>
-      <c r="D29" s="324"/>
-      <c r="E29" s="324"/>
-      <c r="F29" s="324"/>
-      <c r="G29" s="324"/>
-      <c r="H29" s="325"/>
+      <c r="C29" s="566"/>
+      <c r="D29" s="566"/>
+      <c r="E29" s="566"/>
+      <c r="F29" s="566"/>
+      <c r="G29" s="566"/>
+      <c r="H29" s="567"/>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
@@ -25652,12 +25277,12 @@
     <row r="30" ht="23.1" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" s="322"/>
       <c r="B30" s="323"/>
-      <c r="C30" s="324"/>
-      <c r="D30" s="324"/>
-      <c r="E30" s="324"/>
-      <c r="F30" s="324"/>
-      <c r="G30" s="324"/>
-      <c r="H30" s="325"/>
+      <c r="C30" s="566"/>
+      <c r="D30" s="566"/>
+      <c r="E30" s="566"/>
+      <c r="F30" s="566"/>
+      <c r="G30" s="566"/>
+      <c r="H30" s="567"/>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
@@ -25679,12 +25304,12 @@
     <row r="31" ht="23.1" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31" s="326"/>
       <c r="B31" s="327"/>
-      <c r="C31" s="328"/>
-      <c r="D31" s="328"/>
-      <c r="E31" s="328"/>
-      <c r="F31" s="328"/>
-      <c r="G31" s="328"/>
-      <c r="H31" s="329"/>
+      <c r="C31" s="568"/>
+      <c r="D31" s="568"/>
+      <c r="E31" s="568"/>
+      <c r="F31" s="568"/>
+      <c r="G31" s="568"/>
+      <c r="H31" s="569"/>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>

</xml_diff>